<commit_message>
UI improvements, fixed Tesseract paths, and added database export feature
</commit_message>
<xml_diff>
--- a/data/extracted/business_cards.xlsx
+++ b/data/extracted/business_cards.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,6 +652,71 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mehender Banga</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MAYA SALES HITACHI,</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>mayasales.hissar@gmail.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>+919215329586</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Plot No. 4, Ground Floor, Near Reliance Fresh Plot No. 4, Ground Floor, Near Reliance Fresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Prop Satish Kumar Saini</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ho IN29) ‘Sale &amp; Repair _</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>8901260152, 9812610152</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>_ fanguard ee fe Iy- ache _ Linguard fe fe I- -Ee</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C Sdiohet</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>check raw content</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>